<commit_message>
fix: limite affichage produits 50 max (titre affiche total + note)
</commit_message>
<xml_diff>
--- a/outputs/facture_B2613862_02-05-2026.xlsx
+++ b/outputs/facture_B2613862_02-05-2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AC2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,90 +471,105 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>timbre_fiscal</t>
+          <t>net_a_payer</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>net_a_payer</t>
+          <t>devise</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>devise</t>
+          <t>Bon de Livraison</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Siège Social</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Téléphone</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Télécopie</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Site Web</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Bon de Livraison</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>TVA19 Montant</t>
+          <t>Code client</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>TVA19 TVA</t>
+          <t>Client Nom</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
+          <t>Client Adresse</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Client Tel</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Client MF</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
           <t>Total Brut HT</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Total Remise</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Total TVA</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Net à Payer</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>ARRETE A LA SOMME DE</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Montant en lettres</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>remarque</t>
         </is>
@@ -573,12 +588,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TOP ETANCHETIE</t>
+          <t>TOP ETANCHEITE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>76, Rue 18 Janvier 1952, 1000 Tunis - Tunisie</t>
+          <t>Siège Social : 76, Rue 18 Janvier 1952, 1000 Tunis - Tunisie</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -595,78 +610,99 @@
         <v>582.548</v>
       </c>
       <c r="H2" t="n">
-        <v>110.687</v>
+        <v>110.684</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
         <v>693.232</v>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>TND</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>TND</t>
+          <t>B2613862</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>76, Rue 18 Janvier 1952, 1000 Tunis - Tunisie</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>+216 71 350 228</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>+216 71 350 228</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>contact@top-etancheite.com</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>www.top-etancheite.com</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>432555DAM000</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>B2613862</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>02/05/2026</t>
-        </is>
-      </c>
-      <c r="S2" t="n">
-        <v>582.548</v>
-      </c>
-      <c r="T2" t="n">
-        <v>110.687</v>
-      </c>
-      <c r="U2" t="n">
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>014937</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>STE YAK INDUSTRY</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>76 S1 AV INDEPENDANCE MENZEL BOURGUIBA 7050</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>98 992 646</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>1837131S</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
         <v>728.1849999999999</v>
       </c>
-      <c r="V2" t="n">
+      <c r="Y2" t="n">
         <v>145.637</v>
       </c>
-      <c r="W2" t="n">
-        <v>110.687</v>
-      </c>
-      <c r="X2" t="n">
+      <c r="Z2" t="n">
+        <v>110.684</v>
+      </c>
+      <c r="AA2" t="n">
         <v>693.232</v>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>SIX CENT QUATRE VINGT TREIZE DINARS DEUX CENT TRENTE DEUX MILLIMES</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Rien à signaler</t>
         </is>
@@ -724,22 +760,22 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Nom Client</t>
+          <t>Nom du client</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Adresse Client</t>
+          <t>Adresse du client</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Tel Client</t>
+          <t>Téléphone du client</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>MF Client</t>
+          <t>MF du client</t>
         </is>
       </c>
     </row>
@@ -886,7 +922,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>JOINT TORIQUE EN NBR70 OR 053-6</t>
+          <t>JOINT TORIQUE EN NBR70 OR 53-6</t>
         </is>
       </c>
       <c r="C3" t="n">

</xml_diff>